<commit_message>
class diagram-> use case -> SADD -> html design
</commit_message>
<xml_diff>
--- a/requirements/BRS_IEEE29148_Checklist.xlsx
+++ b/requirements/BRS_IEEE29148_Checklist.xlsx
@@ -623,7 +623,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>requirements/BRD_IP_Camera_Web.md – phiên bản 0.3</t>
+          <t>requirements/BRD_IP_Camera_Web.md – phiên bản 0.5</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Các dòng đã được điền sẵn kết quả rà soát BRS v0.3 và có thể dùng làm mẫu cho các lần rà soát sau.</t>
+          <t>Các dòng đã được điền sẵn kết quả rà soát BRS v0.5 và có thể dùng làm mẫu cho các lần rà soát sau.</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3720,7 @@
       </c>
       <c r="H53" s="20" t="inlineStr">
         <is>
-          <t>Ma trận truy vết bao phủ BO-01 đến BO-05, P1 đến P5, BR-01 đến BR-38.</t>
+          <t>Ma trận truy vết bao phủ BO-01 đến BO-05, P1 đến P5, BR-01 đến BR-40.</t>
         </is>
       </c>
       <c r="I53" s="20" t="n"/>

</xml_diff>